<commit_message>
feat(transmitters): adapt bulk upload model to transmitter & bird info and add Reception Date column
</commit_message>
<xml_diff>
--- a/public/templates/HBTrack_Transmitters_Bulk_Upload_Template.xlsx
+++ b/public/templates/HBTrack_Transmitters_Bulk_Upload_Template.xlsx
@@ -398,23 +398,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:Y2"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" customWidth="1"/>
-    <col min="2" max="2" width="25.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="24.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
     <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="20.83203125" customWidth="1"/>
-    <col min="11" max="11" width="8.83203125" customWidth="1"/>
-    <col min="12" max="12" width="12.83203125" customWidth="1"/>
-    <col min="13" max="13" width="14.83203125" customWidth="1"/>
-    <col min="14" max="14" width="14.83203125" customWidth="1"/>
-    <col min="15" max="15" width="35.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="20.83203125" customWidth="1"/>
+    <col min="12" max="12" width="16.83203125" customWidth="1"/>
+    <col min="13" max="13" width="18.83203125" customWidth="1"/>
+    <col min="14" max="14" width="16.83203125" customWidth="1"/>
+    <col min="15" max="15" width="12.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="16.83203125" customWidth="1"/>
+    <col min="18" max="18" width="20.83203125" customWidth="1"/>
+    <col min="19" max="19" width="8.83203125" customWidth="1"/>
+    <col min="20" max="20" width="12.83203125" customWidth="1"/>
+    <col min="21" max="21" width="14.83203125" customWidth="1"/>
+    <col min="22" max="22" width="14.83203125" customWidth="1"/>
+    <col min="23" max="23" width="14.83203125" customWidth="1"/>
+    <col min="24" max="24" width="14.83203125" customWidth="1"/>
+    <col min="25" max="25" width="35.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -422,45 +432,75 @@
         <v>ptt_id *</v>
       </c>
       <c r="B1" t="str">
+        <v>frequency</v>
+      </c>
+      <c r="C1" t="str">
+        <v>hex_id</v>
+      </c>
+      <c r="D1" t="str">
         <v>transmitter_model *</v>
       </c>
-      <c r="C1" t="str">
+      <c r="E1" t="str">
         <v>manufacturer</v>
       </c>
-      <c r="D1" t="str">
+      <c r="F1" t="str">
+        <v>reception_date</v>
+      </c>
+      <c r="G1" t="str">
+        <v>status *</v>
+      </c>
+      <c r="H1" t="str">
+        <v>deployed</v>
+      </c>
+      <c r="I1" t="str">
+        <v>site_location</v>
+      </c>
+      <c r="J1" t="str">
+        <v>program_region</v>
+      </c>
+      <c r="K1" t="str">
+        <v>satellite_time</v>
+      </c>
+      <c r="L1" t="str">
+        <v>radio_time</v>
+      </c>
+      <c r="M1" t="str">
+        <v>duty_cycle</v>
+      </c>
+      <c r="N1" t="str">
         <v>serial_number</v>
       </c>
-      <c r="E1" t="str">
+      <c r="O1" t="str">
         <v>weight_g</v>
       </c>
-      <c r="F1" t="str">
-        <v>status *</v>
-      </c>
-      <c r="G1" t="str">
-        <v>duty_cycle</v>
-      </c>
-      <c r="H1" t="str">
-        <v>deployment_date</v>
-      </c>
-      <c r="I1" t="str">
+      <c r="P1" t="str">
         <v>bird_ring_number</v>
       </c>
-      <c r="J1" t="str">
+      <c r="Q1" t="str">
+        <v>darvic_number</v>
+      </c>
+      <c r="R1" t="str">
         <v>species</v>
       </c>
-      <c r="K1" t="str">
+      <c r="S1" t="str">
         <v>sex</v>
       </c>
-      <c r="L1" t="str">
+      <c r="T1" t="str">
         <v>origin</v>
       </c>
-      <c r="M1" t="str">
+      <c r="U1" t="str">
+        <v>hatch_date</v>
+      </c>
+      <c r="V1" t="str">
+        <v>release_date</v>
+      </c>
+      <c r="W1" t="str">
         <v>release_lat</v>
       </c>
-      <c r="N1" t="str">
+      <c r="X1" t="str">
         <v>release_lon</v>
       </c>
-      <c r="O1" t="str">
+      <c r="Y1" t="str">
         <v>notes</v>
       </c>
     </row>
@@ -469,302 +509,477 @@
         <v>244289</v>
       </c>
       <c r="B2" t="str">
+        <v>401.650</v>
+      </c>
+      <c r="C2" t="str">
+        <v>112A3F</v>
+      </c>
+      <c r="D2" t="str">
         <v>Solar Argos/GPS PTT</v>
       </c>
-      <c r="C2" t="str">
+      <c r="E2" t="str">
         <v>Microwave Telemetry</v>
       </c>
-      <c r="D2" t="str">
+      <c r="F2" t="str">
+        <v>2024-01-15</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Active</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Al Ain Desert</v>
+      </c>
+      <c r="J2" t="str">
+        <v>UAE East</v>
+      </c>
+      <c r="K2" t="str">
+        <v>10h ON / 24h OFF</v>
+      </c>
+      <c r="L2" t="str">
+        <v>12:00 - 18:00</v>
+      </c>
+      <c r="M2" t="str">
+        <v>10h ON / 24h OFF</v>
+      </c>
+      <c r="N2" t="str">
         <v>SN-244289</v>
       </c>
-      <c r="E2">
+      <c r="O2">
         <v>22</v>
       </c>
-      <c r="F2" t="str">
-        <v>Active</v>
-      </c>
-      <c r="G2" t="str">
-        <v>10h ON / 24h OFF</v>
-      </c>
-      <c r="H2" t="str">
+      <c r="P2" t="str">
+        <v>UA-9982</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>DV-104</v>
+      </c>
+      <c r="R2" t="str">
+        <v>Houbara Bustard</v>
+      </c>
+      <c r="S2" t="str">
+        <v>M</v>
+      </c>
+      <c r="T2" t="str">
+        <v>Breeding</v>
+      </c>
+      <c r="U2" t="str">
+        <v>2023-05-10</v>
+      </c>
+      <c r="V2" t="str">
         <v>2024-03-15</v>
       </c>
-      <c r="I2" t="str">
-        <v>UA-9982</v>
-      </c>
-      <c r="J2" t="str">
-        <v>Houbara Bustard</v>
-      </c>
-      <c r="K2" t="str">
-        <v>M</v>
-      </c>
-      <c r="L2" t="str">
-        <v>Breeding</v>
-      </c>
-      <c r="M2">
+      <c r="W2">
         <v>24.12345</v>
       </c>
-      <c r="N2">
+      <c r="X2">
         <v>54.54321</v>
       </c>
-      <c r="O2" t="str">
+      <c r="Y2" t="str">
         <v>Example row - replace with your data</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Y2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D29"/>
   <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="35.83203125" customWidth="1"/>
-    <col min="4" max="4" width="45.83203125" customWidth="1"/>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="45.83203125" customWidth="1"/>
+    <col min="4" max="4" width="60.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>HBTrack — Transmitters Bulk Upload Instructions</v>
+        <v>HBTrack — Transmitters &amp; Birds Bulk Upload Instructions</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>This template allows uploading transmitters and automatically linking or creating associated bird profiles.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Column Name</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Required</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Format / Allowed Values</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Description</v>
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ptt_id</v>
+        <v>Column Name</v>
       </c>
       <c r="B4" t="str">
-        <v>YES</v>
+        <v>Required</v>
       </c>
       <c r="C4" t="str">
-        <v>3-10 digits (e.g. 244289)</v>
+        <v>Format / Allowed Values</v>
       </c>
       <c r="D4" t="str">
-        <v>Unique platform ID of the transmitter.</v>
+        <v>Description</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>transmitter_model</v>
+        <v>ptt_id</v>
       </c>
       <c r="B5" t="str">
         <v>YES</v>
       </c>
       <c r="C5" t="str">
-        <v>Text (e.g. Solar Argos/GPS PTT)</v>
+        <v>3-10 digits (e.g. 244289)</v>
       </c>
       <c r="D5" t="str">
-        <v>Transmitter model.</v>
+        <v>Unique platform ID of the transmitter.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>manufacturer</v>
+        <v>frequency</v>
       </c>
       <c r="B6" t="str">
         <v>No</v>
       </c>
       <c r="C6" t="str">
-        <v>Text (e.g. Microwave Telemetry, North Star)</v>
+        <v>Number/Text (e.g. 401.650)</v>
       </c>
       <c r="D6" t="str">
-        <v>Manufacturer name.</v>
+        <v>Transmission frequency in MHz.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>serial_number</v>
+        <v>hex_id</v>
       </c>
       <c r="B7" t="str">
         <v>No</v>
       </c>
       <c r="C7" t="str">
-        <v>Text</v>
+        <v>Hexadecimal (e.g. 112A3F)</v>
       </c>
       <c r="D7" t="str">
-        <v>Device serial number.</v>
+        <v>Argos Hex ID.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>weight_g</v>
+        <v>transmitter_model</v>
       </c>
       <c r="B8" t="str">
-        <v>No</v>
+        <v>YES</v>
       </c>
       <c r="C8" t="str">
-        <v>Number (e.g. 22)</v>
+        <v>Text (e.g. Solar Argos/GPS PTT, GeoTrack 20g)</v>
       </c>
       <c r="D8" t="str">
-        <v>Weight in grams.</v>
+        <v>Model of the transmitter.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>status</v>
+        <v>manufacturer</v>
       </c>
       <c r="B9" t="str">
-        <v>YES</v>
+        <v>No</v>
       </c>
       <c r="C9" t="str">
-        <v>Active | Inactive | Dead | Static test</v>
+        <v>Text (e.g. Microwave Telemetry, North Star)</v>
       </c>
       <c r="D9" t="str">
-        <v>Device status.</v>
+        <v>Origin company / manufacturer.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>duty_cycle</v>
+        <v>reception_date</v>
       </c>
       <c r="B10" t="str">
         <v>No</v>
       </c>
       <c r="C10" t="str">
-        <v>Text (e.g. 10h ON / 24h OFF)</v>
+        <v>YYYY-MM-DD (e.g. 2024-01-15)</v>
       </c>
       <c r="D10" t="str">
-        <v>Transmission schedule.</v>
+        <v>Date when the transmitter was received.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>deployment_date</v>
+        <v>status</v>
       </c>
       <c r="B11" t="str">
-        <v>No</v>
+        <v>YES</v>
       </c>
       <c r="C11" t="str">
-        <v>YYYY-MM-DD</v>
+        <v>Active | Inactive | Dead | Static test | Potential Mortality</v>
       </c>
       <c r="D11" t="str">
-        <v>Date deployed.</v>
+        <v>Operational status of the transmitter.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>bird_ring_number</v>
+        <v>deployed</v>
       </c>
       <c r="B12" t="str">
         <v>No</v>
       </c>
       <c r="C12" t="str">
-        <v>Text</v>
+        <v>Yes | No (or true / false)</v>
       </c>
       <c r="D12" t="str">
-        <v>Ring number of existing bird to link with.</v>
+        <v>Whether the device is currently deployed on a bird.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>species</v>
+        <v>site_location</v>
       </c>
       <c r="B13" t="str">
         <v>No</v>
       </c>
       <c r="C13" t="str">
-        <v>Text</v>
+        <v>Text (e.g. Al Ain Desert)</v>
       </c>
       <c r="D13" t="str">
-        <v>Default: Houbara Bustard.</v>
+        <v>Deployment site location.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>sex</v>
+        <v>program_region</v>
       </c>
       <c r="B14" t="str">
         <v>No</v>
       </c>
       <c r="C14" t="str">
-        <v>M or F</v>
+        <v>Text (e.g. UAE East, Central Saudi Arabia)</v>
       </c>
       <c r="D14" t="str">
-        <v>Bird gender.</v>
+        <v>Operational program region.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>origin</v>
+        <v>satellite_time</v>
       </c>
       <c r="B15" t="str">
         <v>No</v>
       </c>
       <c r="C15" t="str">
-        <v>Wild or Breeding</v>
+        <v>Text (e.g. 10h ON / 24h OFF, Continuous)</v>
       </c>
       <c r="D15" t="str">
-        <v>Bird origin.</v>
+        <v>Satellite transmission schedule/cycle.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>release_lat</v>
+        <v>radio_time</v>
       </c>
       <c r="B16" t="str">
         <v>No</v>
       </c>
       <c r="C16" t="str">
-        <v>Decimal (-90.0 to 90.0)</v>
+        <v>Text (e.g. 12:00 - 18:00, None)</v>
       </c>
       <c r="D16" t="str">
-        <v>Release latitude.</v>
+        <v>VHF radio beacon transmission time.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>release_lon</v>
+        <v>duty_cycle</v>
       </c>
       <c r="B17" t="str">
         <v>No</v>
       </c>
       <c r="C17" t="str">
-        <v>Decimal (-180.0 to 180.0)</v>
+        <v>Text (e.g. 10h ON / 24h OFF)</v>
       </c>
       <c r="D17" t="str">
-        <v>Release longitude.</v>
+        <v>Transmission schedule duty cycle.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
+        <v>serial_number</v>
+      </c>
+      <c r="B18" t="str">
+        <v>No</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Text (e.g. SN-244289)</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Device hardware serial number.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>weight_g</v>
+      </c>
+      <c r="B19" t="str">
+        <v>No</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Number (e.g. 22)</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Weight of device in grams.</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>bird_ring_number</v>
+      </c>
+      <c r="B20" t="str">
+        <v>No</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Text (e.g. UA-9982)</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Ring ID of existing bird to link, or new bird to register.</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>darvic_number</v>
+      </c>
+      <c r="B21" t="str">
+        <v>No</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Text (e.g. DV-104)</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Colored darvic ring/band code.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>species</v>
+      </c>
+      <c r="B22" t="str">
+        <v>No</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Text (e.g. Houbara Bustard)</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Bird species (defaults to Houbara Bustard).</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>sex</v>
+      </c>
+      <c r="B23" t="str">
+        <v>No</v>
+      </c>
+      <c r="C23" t="str">
+        <v>M | F</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Bird gender/sex.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>origin</v>
+      </c>
+      <c r="B24" t="str">
+        <v>No</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Wild | Breeding</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Origin of the bird.</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>hatch_date</v>
+      </c>
+      <c r="B25" t="str">
+        <v>No</v>
+      </c>
+      <c r="C25" t="str">
+        <v>YYYY-MM-DD (e.g. 2023-05-10)</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Hatch date of bird.</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>release_date</v>
+      </c>
+      <c r="B26" t="str">
+        <v>No</v>
+      </c>
+      <c r="C26" t="str">
+        <v>YYYY-MM-DD (e.g. 2024-03-15)</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Release date of bird / deployment date.</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>release_lat</v>
+      </c>
+      <c r="B27" t="str">
+        <v>No</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Decimal (-90.0 to 90.0)</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Release site latitude.</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>release_lon</v>
+      </c>
+      <c r="B28" t="str">
+        <v>No</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Decimal (-180.0 to 180.0)</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Release site longitude.</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
         <v>notes</v>
       </c>
-      <c r="B18" t="str">
-        <v>No</v>
-      </c>
-      <c r="C18" t="str">
+      <c r="B29" t="str">
+        <v>No</v>
+      </c>
+      <c r="C29" t="str">
         <v>Text</v>
       </c>
-      <c r="D18" t="str">
-        <v>Additional comments.</v>
+      <c r="D29" t="str">
+        <v>Comments and notes about the transmitter and bird.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D29"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(transmitters): make reception_date obligatory (accepts year), replace serial_number with hex_id, add format guide & dynamic template download
</commit_message>
<xml_diff>
--- a/public/templates/HBTrack_Transmitters_Bulk_Upload_Template.xlsx
+++ b/public/templates/HBTrack_Transmitters_Bulk_Upload_Template.xlsx
@@ -398,14 +398,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y2"/>
+  <dimension ref="A1:X2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
     <col min="4" max="4" width="24.83203125" customWidth="1"/>
     <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
     <col min="7" max="7" width="14.83203125" customWidth="1"/>
     <col min="8" max="8" width="12.83203125" customWidth="1"/>
     <col min="9" max="9" width="18.83203125" customWidth="1"/>
@@ -413,18 +413,17 @@
     <col min="11" max="11" width="20.83203125" customWidth="1"/>
     <col min="12" max="12" width="16.83203125" customWidth="1"/>
     <col min="13" max="13" width="18.83203125" customWidth="1"/>
-    <col min="14" max="14" width="16.83203125" customWidth="1"/>
-    <col min="15" max="15" width="12.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="16.83203125" customWidth="1"/>
-    <col min="18" max="18" width="20.83203125" customWidth="1"/>
-    <col min="19" max="19" width="8.83203125" customWidth="1"/>
-    <col min="20" max="20" width="12.83203125" customWidth="1"/>
+    <col min="14" max="14" width="12.83203125" customWidth="1"/>
+    <col min="15" max="15" width="18.83203125" customWidth="1"/>
+    <col min="16" max="16" width="16.83203125" customWidth="1"/>
+    <col min="17" max="17" width="20.83203125" customWidth="1"/>
+    <col min="18" max="18" width="8.83203125" customWidth="1"/>
+    <col min="19" max="19" width="12.83203125" customWidth="1"/>
+    <col min="20" max="20" width="14.83203125" customWidth="1"/>
     <col min="21" max="21" width="14.83203125" customWidth="1"/>
     <col min="22" max="22" width="14.83203125" customWidth="1"/>
     <col min="23" max="23" width="14.83203125" customWidth="1"/>
-    <col min="24" max="24" width="14.83203125" customWidth="1"/>
-    <col min="25" max="25" width="35.83203125" customWidth="1"/>
+    <col min="24" max="24" width="35.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -444,7 +443,7 @@
         <v>manufacturer</v>
       </c>
       <c r="F1" t="str">
-        <v>reception_date</v>
+        <v>reception_date *</v>
       </c>
       <c r="G1" t="str">
         <v>status *</v>
@@ -468,39 +467,36 @@
         <v>duty_cycle</v>
       </c>
       <c r="N1" t="str">
-        <v>serial_number</v>
+        <v>weight_g</v>
       </c>
       <c r="O1" t="str">
-        <v>weight_g</v>
+        <v>bird_ring_number</v>
       </c>
       <c r="P1" t="str">
-        <v>bird_ring_number</v>
+        <v>darvic_number</v>
       </c>
       <c r="Q1" t="str">
-        <v>darvic_number</v>
+        <v>species</v>
       </c>
       <c r="R1" t="str">
-        <v>species</v>
+        <v>sex</v>
       </c>
       <c r="S1" t="str">
-        <v>sex</v>
+        <v>origin</v>
       </c>
       <c r="T1" t="str">
-        <v>origin</v>
+        <v>hatch_date</v>
       </c>
       <c r="U1" t="str">
-        <v>hatch_date</v>
+        <v>release_date</v>
       </c>
       <c r="V1" t="str">
-        <v>release_date</v>
+        <v>release_lat</v>
       </c>
       <c r="W1" t="str">
-        <v>release_lat</v>
+        <v>release_lon</v>
       </c>
       <c r="X1" t="str">
-        <v>release_lon</v>
-      </c>
-      <c r="Y1" t="str">
         <v>notes</v>
       </c>
     </row>
@@ -521,7 +517,7 @@
         <v>Microwave Telemetry</v>
       </c>
       <c r="F2" t="str">
-        <v>2024-01-15</v>
+        <v>2024</v>
       </c>
       <c r="G2" t="str">
         <v>Active</v>
@@ -544,58 +540,55 @@
       <c r="M2" t="str">
         <v>10h ON / 24h OFF</v>
       </c>
-      <c r="N2" t="str">
-        <v>SN-244289</v>
-      </c>
-      <c r="O2">
+      <c r="N2">
         <v>22</v>
       </c>
+      <c r="O2" t="str">
+        <v>UA-9982</v>
+      </c>
       <c r="P2" t="str">
-        <v>UA-9982</v>
+        <v>DV-104</v>
       </c>
       <c r="Q2" t="str">
-        <v>DV-104</v>
+        <v>Houbara Bustard</v>
       </c>
       <c r="R2" t="str">
-        <v>Houbara Bustard</v>
+        <v>M</v>
       </c>
       <c r="S2" t="str">
-        <v>M</v>
+        <v>Breeding</v>
       </c>
       <c r="T2" t="str">
-        <v>Breeding</v>
+        <v>2023-05-10</v>
       </c>
       <c r="U2" t="str">
-        <v>2023-05-10</v>
-      </c>
-      <c r="V2" t="str">
         <v>2024-03-15</v>
       </c>
+      <c r="V2">
+        <v>24.12345</v>
+      </c>
       <c r="W2">
-        <v>24.12345</v>
-      </c>
-      <c r="X2">
         <v>54.54321</v>
       </c>
-      <c r="Y2" t="str">
+      <c r="X2" t="str">
         <v>Example row - replace with your data</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Y2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:X2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D28"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
     <col min="3" max="3" width="45.83203125" customWidth="1"/>
-    <col min="4" max="4" width="60.83203125" customWidth="1"/>
+    <col min="4" max="4" width="65.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -666,7 +659,7 @@
         <v>Hexadecimal (e.g. 112A3F)</v>
       </c>
       <c r="D7" t="str">
-        <v>Argos Hex ID.</v>
+        <v>Argos Hex ID (optional, replaces serial number).</v>
       </c>
     </row>
     <row r="8">
@@ -702,13 +695,13 @@
         <v>reception_date</v>
       </c>
       <c r="B10" t="str">
-        <v>No</v>
+        <v>YES (Obligatory)</v>
       </c>
       <c r="C10" t="str">
-        <v>YYYY-MM-DD (e.g. 2024-01-15)</v>
+        <v>Year (e.g. 2024) or YYYY-MM-DD (e.g. 2024-01-15)</v>
       </c>
       <c r="D10" t="str">
-        <v>Date when the transmitter was received.</v>
+        <v>Reception date: accepts 4-digit year only (e.g. 2024) or full date.</v>
       </c>
     </row>
     <row r="11">
@@ -811,175 +804,161 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>serial_number</v>
+        <v>weight_g</v>
       </c>
       <c r="B18" t="str">
         <v>No</v>
       </c>
       <c r="C18" t="str">
-        <v>Text (e.g. SN-244289)</v>
+        <v>Number (e.g. 22)</v>
       </c>
       <c r="D18" t="str">
-        <v>Device hardware serial number.</v>
+        <v>Weight of device in grams.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>weight_g</v>
+        <v>bird_ring_number</v>
       </c>
       <c r="B19" t="str">
         <v>No</v>
       </c>
       <c r="C19" t="str">
-        <v>Number (e.g. 22)</v>
+        <v>Text (e.g. UA-9982)</v>
       </c>
       <c r="D19" t="str">
-        <v>Weight of device in grams.</v>
+        <v>Ring ID of existing bird to link, or new bird to register.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>bird_ring_number</v>
+        <v>darvic_number</v>
       </c>
       <c r="B20" t="str">
         <v>No</v>
       </c>
       <c r="C20" t="str">
-        <v>Text (e.g. UA-9982)</v>
+        <v>Text (e.g. DV-104)</v>
       </c>
       <c r="D20" t="str">
-        <v>Ring ID of existing bird to link, or new bird to register.</v>
+        <v>Colored darvic ring/band code.</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>darvic_number</v>
+        <v>species</v>
       </c>
       <c r="B21" t="str">
         <v>No</v>
       </c>
       <c r="C21" t="str">
-        <v>Text (e.g. DV-104)</v>
+        <v>Text (e.g. Houbara Bustard)</v>
       </c>
       <c r="D21" t="str">
-        <v>Colored darvic ring/band code.</v>
+        <v>Bird species (defaults to Houbara Bustard).</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>species</v>
+        <v>sex</v>
       </c>
       <c r="B22" t="str">
         <v>No</v>
       </c>
       <c r="C22" t="str">
-        <v>Text (e.g. Houbara Bustard)</v>
+        <v>M | F</v>
       </c>
       <c r="D22" t="str">
-        <v>Bird species (defaults to Houbara Bustard).</v>
+        <v>Bird gender/sex.</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>sex</v>
+        <v>origin</v>
       </c>
       <c r="B23" t="str">
         <v>No</v>
       </c>
       <c r="C23" t="str">
-        <v>M | F</v>
+        <v>Wild | Breeding</v>
       </c>
       <c r="D23" t="str">
-        <v>Bird gender/sex.</v>
+        <v>Origin of the bird.</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>origin</v>
+        <v>hatch_date</v>
       </c>
       <c r="B24" t="str">
         <v>No</v>
       </c>
       <c r="C24" t="str">
-        <v>Wild | Breeding</v>
+        <v>YYYY-MM-DD (e.g. 2023-05-10)</v>
       </c>
       <c r="D24" t="str">
-        <v>Origin of the bird.</v>
+        <v>Hatch date of bird.</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>hatch_date</v>
+        <v>release_date</v>
       </c>
       <c r="B25" t="str">
         <v>No</v>
       </c>
       <c r="C25" t="str">
-        <v>YYYY-MM-DD (e.g. 2023-05-10)</v>
+        <v>YYYY-MM-DD (e.g. 2024-03-15)</v>
       </c>
       <c r="D25" t="str">
-        <v>Hatch date of bird.</v>
+        <v>Release date of bird / deployment date.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>release_date</v>
+        <v>release_lat</v>
       </c>
       <c r="B26" t="str">
         <v>No</v>
       </c>
       <c r="C26" t="str">
-        <v>YYYY-MM-DD (e.g. 2024-03-15)</v>
+        <v>Decimal (-90.0 to 90.0)</v>
       </c>
       <c r="D26" t="str">
-        <v>Release date of bird / deployment date.</v>
+        <v>Release site latitude.</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>release_lat</v>
+        <v>release_lon</v>
       </c>
       <c r="B27" t="str">
         <v>No</v>
       </c>
       <c r="C27" t="str">
-        <v>Decimal (-90.0 to 90.0)</v>
+        <v>Decimal (-180.0 to 180.0)</v>
       </c>
       <c r="D27" t="str">
-        <v>Release site latitude.</v>
+        <v>Release site longitude.</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>release_lon</v>
+        <v>notes</v>
       </c>
       <c r="B28" t="str">
         <v>No</v>
       </c>
       <c r="C28" t="str">
-        <v>Decimal (-180.0 to 180.0)</v>
+        <v>Text</v>
       </c>
       <c r="D28" t="str">
-        <v>Release site longitude.</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>notes</v>
-      </c>
-      <c r="B29" t="str">
-        <v>No</v>
-      </c>
-      <c r="C29" t="str">
-        <v>Text</v>
-      </c>
-      <c r="D29" t="str">
         <v>Comments and notes about the transmitter and bird.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D28"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(transmitters): align Excel model to 16 columns replacing serial_number with hex_id, add reception_date, and update format guide
</commit_message>
<xml_diff>
--- a/public/templates/HBTrack_Transmitters_Bulk_Upload_Template.xlsx
+++ b/public/templates/HBTrack_Transmitters_Bulk_Upload_Template.xlsx
@@ -398,32 +398,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X2"/>
+  <dimension ref="A1:P2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
     <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="16.83203125" customWidth="1"/>
     <col min="10" max="10" width="18.83203125" customWidth="1"/>
     <col min="11" max="11" width="20.83203125" customWidth="1"/>
-    <col min="12" max="12" width="16.83203125" customWidth="1"/>
-    <col min="13" max="13" width="18.83203125" customWidth="1"/>
-    <col min="14" max="14" width="12.83203125" customWidth="1"/>
-    <col min="15" max="15" width="18.83203125" customWidth="1"/>
-    <col min="16" max="16" width="16.83203125" customWidth="1"/>
-    <col min="17" max="17" width="20.83203125" customWidth="1"/>
-    <col min="18" max="18" width="8.83203125" customWidth="1"/>
-    <col min="19" max="19" width="12.83203125" customWidth="1"/>
-    <col min="20" max="20" width="14.83203125" customWidth="1"/>
-    <col min="21" max="21" width="14.83203125" customWidth="1"/>
-    <col min="22" max="22" width="14.83203125" customWidth="1"/>
-    <col min="23" max="23" width="14.83203125" customWidth="1"/>
-    <col min="24" max="24" width="35.83203125" customWidth="1"/>
+    <col min="12" max="12" width="8.83203125" customWidth="1"/>
+    <col min="13" max="13" width="12.83203125" customWidth="1"/>
+    <col min="14" max="14" width="14.83203125" customWidth="1"/>
+    <col min="15" max="15" width="14.83203125" customWidth="1"/>
+    <col min="16" max="16" width="35.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -431,72 +423,48 @@
         <v>ptt_id *</v>
       </c>
       <c r="B1" t="str">
-        <v>frequency</v>
+        <v>transmitter_model *</v>
       </c>
       <c r="C1" t="str">
+        <v>manufacturer</v>
+      </c>
+      <c r="D1" t="str">
         <v>hex_id</v>
       </c>
-      <c r="D1" t="str">
-        <v>transmitter_model *</v>
-      </c>
       <c r="E1" t="str">
-        <v>manufacturer</v>
+        <v>reception_date *</v>
       </c>
       <c r="F1" t="str">
-        <v>reception_date *</v>
+        <v>weight_g</v>
       </c>
       <c r="G1" t="str">
         <v>status *</v>
       </c>
       <c r="H1" t="str">
-        <v>deployed</v>
+        <v>duty_cycle</v>
       </c>
       <c r="I1" t="str">
-        <v>site_location</v>
+        <v>deployment_date</v>
       </c>
       <c r="J1" t="str">
-        <v>program_region</v>
+        <v>bird_ring_number</v>
       </c>
       <c r="K1" t="str">
-        <v>satellite_time</v>
+        <v>species</v>
       </c>
       <c r="L1" t="str">
-        <v>radio_time</v>
+        <v>sex</v>
       </c>
       <c r="M1" t="str">
-        <v>duty_cycle</v>
+        <v>origin</v>
       </c>
       <c r="N1" t="str">
-        <v>weight_g</v>
+        <v>release_lat</v>
       </c>
       <c r="O1" t="str">
-        <v>bird_ring_number</v>
+        <v>release_lon</v>
       </c>
       <c r="P1" t="str">
-        <v>darvic_number</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>species</v>
-      </c>
-      <c r="R1" t="str">
-        <v>sex</v>
-      </c>
-      <c r="S1" t="str">
-        <v>origin</v>
-      </c>
-      <c r="T1" t="str">
-        <v>hatch_date</v>
-      </c>
-      <c r="U1" t="str">
-        <v>release_date</v>
-      </c>
-      <c r="V1" t="str">
-        <v>release_lat</v>
-      </c>
-      <c r="W1" t="str">
-        <v>release_lon</v>
-      </c>
-      <c r="X1" t="str">
         <v>notes</v>
       </c>
     </row>
@@ -505,147 +473,132 @@
         <v>244289</v>
       </c>
       <c r="B2" t="str">
-        <v>401.650</v>
+        <v>Solar Argos/GPS PTT</v>
       </c>
       <c r="C2" t="str">
+        <v>Microwave Telemetry</v>
+      </c>
+      <c r="D2" t="str">
         <v>112A3F</v>
       </c>
-      <c r="D2" t="str">
-        <v>Solar Argos/GPS PTT</v>
-      </c>
       <c r="E2" t="str">
-        <v>Microwave Telemetry</v>
-      </c>
-      <c r="F2" t="str">
         <v>2024</v>
+      </c>
+      <c r="F2">
+        <v>22</v>
       </c>
       <c r="G2" t="str">
         <v>Active</v>
       </c>
       <c r="H2" t="str">
-        <v>Yes</v>
+        <v>10h ON / 24h OFF</v>
       </c>
       <c r="I2" t="str">
-        <v>Al Ain Desert</v>
+        <v>2024-03-15</v>
       </c>
       <c r="J2" t="str">
-        <v>UAE East</v>
+        <v>UA-9982</v>
       </c>
       <c r="K2" t="str">
-        <v>10h ON / 24h OFF</v>
+        <v>Houbara Bustard</v>
       </c>
       <c r="L2" t="str">
-        <v>12:00 - 18:00</v>
+        <v>M</v>
       </c>
       <c r="M2" t="str">
-        <v>10h ON / 24h OFF</v>
+        <v>Breeding</v>
       </c>
       <c r="N2">
-        <v>22</v>
-      </c>
-      <c r="O2" t="str">
-        <v>UA-9982</v>
+        <v>24.12345</v>
+      </c>
+      <c r="O2">
+        <v>54.54321</v>
       </c>
       <c r="P2" t="str">
-        <v>DV-104</v>
-      </c>
-      <c r="Q2" t="str">
-        <v>Houbara Bustard</v>
-      </c>
-      <c r="R2" t="str">
-        <v>M</v>
-      </c>
-      <c r="S2" t="str">
-        <v>Breeding</v>
-      </c>
-      <c r="T2" t="str">
-        <v>2023-05-10</v>
-      </c>
-      <c r="U2" t="str">
-        <v>2024-03-15</v>
-      </c>
-      <c r="V2">
-        <v>24.12345</v>
-      </c>
-      <c r="W2">
-        <v>54.54321</v>
-      </c>
-      <c r="X2" t="str">
         <v>Example row - replace with your data</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:X2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D19"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
     <col min="3" max="3" width="45.83203125" customWidth="1"/>
     <col min="4" max="4" width="65.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>HBTrack — Transmitters &amp; Birds Bulk Upload Instructions</v>
+        <v>HBTrack — Transmitters Bulk Upload Instructions</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>This template allows uploading transmitters and automatically linking or creating associated bird profiles.</v>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v/>
+        <v>Column Name</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Required</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Format / Allowed Values</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Description</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Column Name</v>
+        <v>ptt_id</v>
       </c>
       <c r="B4" t="str">
-        <v>Required</v>
+        <v>YES</v>
       </c>
       <c r="C4" t="str">
-        <v>Format / Allowed Values</v>
+        <v>3-10 digits (e.g. 244289)</v>
       </c>
       <c r="D4" t="str">
-        <v>Description</v>
+        <v>Unique platform ID of the transmitter.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ptt_id</v>
+        <v>transmitter_model</v>
       </c>
       <c r="B5" t="str">
         <v>YES</v>
       </c>
       <c r="C5" t="str">
-        <v>3-10 digits (e.g. 244289)</v>
+        <v>Text (e.g. Solar Argos/GPS PTT)</v>
       </c>
       <c r="D5" t="str">
-        <v>Unique platform ID of the transmitter.</v>
+        <v>Transmitter model.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>frequency</v>
+        <v>manufacturer</v>
       </c>
       <c r="B6" t="str">
         <v>No</v>
       </c>
       <c r="C6" t="str">
-        <v>Number/Text (e.g. 401.650)</v>
+        <v>Text (e.g. Microwave Telemetry, North Star)</v>
       </c>
       <c r="D6" t="str">
-        <v>Transmission frequency in MHz.</v>
+        <v>Manufacturer name.</v>
       </c>
     </row>
     <row r="7">
@@ -664,301 +617,175 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>transmitter_model</v>
+        <v>reception_date</v>
       </c>
       <c r="B8" t="str">
         <v>YES</v>
       </c>
       <c r="C8" t="str">
-        <v>Text (e.g. Solar Argos/GPS PTT, GeoTrack 20g)</v>
+        <v>Year (e.g. 2024) or YYYY-MM-DD</v>
       </c>
       <c r="D8" t="str">
-        <v>Model of the transmitter.</v>
+        <v>Date transmitter was received (obligatory, can accept only year).</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>manufacturer</v>
+        <v>weight_g</v>
       </c>
       <c r="B9" t="str">
         <v>No</v>
       </c>
       <c r="C9" t="str">
-        <v>Text (e.g. Microwave Telemetry, North Star)</v>
+        <v>Number (e.g. 22)</v>
       </c>
       <c r="D9" t="str">
-        <v>Origin company / manufacturer.</v>
+        <v>Weight in grams.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>reception_date</v>
+        <v>status</v>
       </c>
       <c r="B10" t="str">
-        <v>YES (Obligatory)</v>
+        <v>YES</v>
       </c>
       <c r="C10" t="str">
-        <v>Year (e.g. 2024) or YYYY-MM-DD (e.g. 2024-01-15)</v>
+        <v>Active | Inactive | Dead | Static test</v>
       </c>
       <c r="D10" t="str">
-        <v>Reception date: accepts 4-digit year only (e.g. 2024) or full date.</v>
+        <v>Device status.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>status</v>
+        <v>duty_cycle</v>
       </c>
       <c r="B11" t="str">
-        <v>YES</v>
+        <v>No</v>
       </c>
       <c r="C11" t="str">
-        <v>Active | Inactive | Dead | Static test | Potential Mortality</v>
+        <v>Text (e.g. 10h ON / 24h OFF)</v>
       </c>
       <c r="D11" t="str">
-        <v>Operational status of the transmitter.</v>
+        <v>Transmission schedule.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>deployed</v>
+        <v>deployment_date</v>
       </c>
       <c r="B12" t="str">
         <v>No</v>
       </c>
       <c r="C12" t="str">
-        <v>Yes | No (or true / false)</v>
+        <v>YYYY-MM-DD</v>
       </c>
       <c r="D12" t="str">
-        <v>Whether the device is currently deployed on a bird.</v>
+        <v>Date deployed.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>site_location</v>
+        <v>bird_ring_number</v>
       </c>
       <c r="B13" t="str">
         <v>No</v>
       </c>
       <c r="C13" t="str">
-        <v>Text (e.g. Al Ain Desert)</v>
+        <v>Text</v>
       </c>
       <c r="D13" t="str">
-        <v>Deployment site location.</v>
+        <v>Ring number of existing bird to link with.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>program_region</v>
+        <v>species</v>
       </c>
       <c r="B14" t="str">
         <v>No</v>
       </c>
       <c r="C14" t="str">
-        <v>Text (e.g. UAE East, Central Saudi Arabia)</v>
+        <v>Text</v>
       </c>
       <c r="D14" t="str">
-        <v>Operational program region.</v>
+        <v>Default: Houbara Bustard.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>satellite_time</v>
+        <v>sex</v>
       </c>
       <c r="B15" t="str">
         <v>No</v>
       </c>
       <c r="C15" t="str">
-        <v>Text (e.g. 10h ON / 24h OFF, Continuous)</v>
+        <v>M or F</v>
       </c>
       <c r="D15" t="str">
-        <v>Satellite transmission schedule/cycle.</v>
+        <v>Bird gender.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>radio_time</v>
+        <v>origin</v>
       </c>
       <c r="B16" t="str">
         <v>No</v>
       </c>
       <c r="C16" t="str">
-        <v>Text (e.g. 12:00 - 18:00, None)</v>
+        <v>Wild or Breeding</v>
       </c>
       <c r="D16" t="str">
-        <v>VHF radio beacon transmission time.</v>
+        <v>Bird origin.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>duty_cycle</v>
+        <v>release_lat</v>
       </c>
       <c r="B17" t="str">
         <v>No</v>
       </c>
       <c r="C17" t="str">
-        <v>Text (e.g. 10h ON / 24h OFF)</v>
+        <v>Decimal (-90.0 to 90.0)</v>
       </c>
       <c r="D17" t="str">
-        <v>Transmission schedule duty cycle.</v>
+        <v>Release latitude.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>weight_g</v>
+        <v>release_lon</v>
       </c>
       <c r="B18" t="str">
         <v>No</v>
       </c>
       <c r="C18" t="str">
-        <v>Number (e.g. 22)</v>
+        <v>Decimal (-180.0 to 180.0)</v>
       </c>
       <c r="D18" t="str">
-        <v>Weight of device in grams.</v>
+        <v>Release longitude.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>bird_ring_number</v>
+        <v>notes</v>
       </c>
       <c r="B19" t="str">
         <v>No</v>
       </c>
       <c r="C19" t="str">
-        <v>Text (e.g. UA-9982)</v>
+        <v>Text</v>
       </c>
       <c r="D19" t="str">
-        <v>Ring ID of existing bird to link, or new bird to register.</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>darvic_number</v>
-      </c>
-      <c r="B20" t="str">
-        <v>No</v>
-      </c>
-      <c r="C20" t="str">
-        <v>Text (e.g. DV-104)</v>
-      </c>
-      <c r="D20" t="str">
-        <v>Colored darvic ring/band code.</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>species</v>
-      </c>
-      <c r="B21" t="str">
-        <v>No</v>
-      </c>
-      <c r="C21" t="str">
-        <v>Text (e.g. Houbara Bustard)</v>
-      </c>
-      <c r="D21" t="str">
-        <v>Bird species (defaults to Houbara Bustard).</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>sex</v>
-      </c>
-      <c r="B22" t="str">
-        <v>No</v>
-      </c>
-      <c r="C22" t="str">
-        <v>M | F</v>
-      </c>
-      <c r="D22" t="str">
-        <v>Bird gender/sex.</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>origin</v>
-      </c>
-      <c r="B23" t="str">
-        <v>No</v>
-      </c>
-      <c r="C23" t="str">
-        <v>Wild | Breeding</v>
-      </c>
-      <c r="D23" t="str">
-        <v>Origin of the bird.</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>hatch_date</v>
-      </c>
-      <c r="B24" t="str">
-        <v>No</v>
-      </c>
-      <c r="C24" t="str">
-        <v>YYYY-MM-DD (e.g. 2023-05-10)</v>
-      </c>
-      <c r="D24" t="str">
-        <v>Hatch date of bird.</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>release_date</v>
-      </c>
-      <c r="B25" t="str">
-        <v>No</v>
-      </c>
-      <c r="C25" t="str">
-        <v>YYYY-MM-DD (e.g. 2024-03-15)</v>
-      </c>
-      <c r="D25" t="str">
-        <v>Release date of bird / deployment date.</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>release_lat</v>
-      </c>
-      <c r="B26" t="str">
-        <v>No</v>
-      </c>
-      <c r="C26" t="str">
-        <v>Decimal (-90.0 to 90.0)</v>
-      </c>
-      <c r="D26" t="str">
-        <v>Release site latitude.</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>release_lon</v>
-      </c>
-      <c r="B27" t="str">
-        <v>No</v>
-      </c>
-      <c r="C27" t="str">
-        <v>Decimal (-180.0 to 180.0)</v>
-      </c>
-      <c r="D27" t="str">
-        <v>Release site longitude.</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>notes</v>
-      </c>
-      <c r="B28" t="str">
-        <v>No</v>
-      </c>
-      <c r="C28" t="str">
-        <v>Text</v>
-      </c>
-      <c r="D28" t="str">
-        <v>Comments and notes about the transmitter and bird.</v>
+        <v>Additional comments.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D19"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>